<commit_message>
deploy: auto-publish via publish-to-github.bat
</commit_message>
<xml_diff>
--- a/法宝属性.xlsx
+++ b/法宝属性.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\背包排列工具\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BackpackArrangementTool\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="12080" activeTab="5"/>
+    <workbookView windowHeight="17775" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="金" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">水!$A$1:$K$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">火!$A$1:$K$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">土!$A$1:$K$47</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">雷!$A$1:$K$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">雷!$A$1:$K$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">体!$A$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -1302,9 +1302,8 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
   </cellXfs>
@@ -1691,7 +1690,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L48"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.6666666666667" customWidth="1"/>
     <col min="2" max="2" width="22.75" customWidth="1"/>
@@ -3340,7 +3339,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A34:K44 A45 C45:K45 I32:K32 A32:G32 A1:K31 A46:G46 K46" numberStoredAsText="1"/>
+    <ignoredError sqref="K46 A46:G46 A1:K31 A32:G32 I32:K32 C45:K45 A45 A34:K44" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3349,7 +3348,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L47"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.6666666666667" customWidth="1"/>
     <col min="2" max="2" width="17.25" customWidth="1"/>
@@ -4992,7 +4991,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:K47 A48:L49" numberStoredAsText="1"/>
+    <ignoredError sqref="A48:L49 A1:K47" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5001,7 +5000,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L47"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.6666666666667" customWidth="1"/>
     <col min="2" max="2" width="17.25" customWidth="1"/>
@@ -6653,7 +6652,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L47"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.6666666666667" customWidth="1"/>
     <col min="2" max="2" width="22.75" customWidth="1"/>
@@ -8304,10 +8303,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L47"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.6666666666667" customWidth="1"/>
-    <col min="2" max="2" width="23.9166666666667" style="3" customWidth="1"/>
+    <col min="2" max="2" width="23.9166666666667" style="2" customWidth="1"/>
     <col min="3" max="4" width="7.41666666666667" customWidth="1"/>
     <col min="5" max="5" width="5.41666666666667" customWidth="1"/>
     <col min="6" max="7" width="7.41666666666667" customWidth="1"/>
@@ -8320,7 +8319,7 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
@@ -8358,7 +8357,7 @@
       <c r="A2" t="s">
         <v>124</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C2">
@@ -8492,7 +8491,7 @@
       <c r="A6" t="s">
         <v>125</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C6">
@@ -8626,7 +8625,7 @@
       <c r="A10" t="s">
         <v>126</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C10">
@@ -8760,7 +8759,7 @@
       <c r="A14" t="s">
         <v>127</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C14">
@@ -8894,7 +8893,7 @@
       <c r="A18" t="s">
         <v>128</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C18">
@@ -8932,7 +8931,7 @@
       <c r="A19" t="s">
         <v>129</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="2" t="s">
         <v>38</v>
       </c>
       <c r="C19">
@@ -9066,7 +9065,7 @@
       <c r="A23" t="s">
         <v>131</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="2" t="s">
         <v>38</v>
       </c>
       <c r="C23">
@@ -9200,7 +9199,7 @@
       <c r="A27" t="s">
         <v>132</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="2" t="s">
         <v>38</v>
       </c>
       <c r="C27">
@@ -9238,7 +9237,7 @@
       <c r="A28" t="s">
         <v>133</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="2" t="s">
         <v>70</v>
       </c>
       <c r="C28">
@@ -9372,7 +9371,7 @@
       <c r="A32" t="s">
         <v>134</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="2" t="s">
         <v>70</v>
       </c>
       <c r="C32">
@@ -9410,7 +9409,7 @@
       <c r="A33" t="s">
         <v>135</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="2" t="s">
         <v>45</v>
       </c>
       <c r="C33">
@@ -9544,7 +9543,7 @@
       <c r="A37" t="s">
         <v>136</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="2" t="s">
         <v>45</v>
       </c>
       <c r="C37">
@@ -9582,7 +9581,7 @@
       <c r="A38" t="s">
         <v>137</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" s="2" t="s">
         <v>45</v>
       </c>
       <c r="C38">
@@ -9620,7 +9619,7 @@
       <c r="A39" t="s">
         <v>138</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B39" s="2" t="s">
         <v>48</v>
       </c>
       <c r="C39">
@@ -9754,7 +9753,7 @@
       <c r="A43" t="s">
         <v>139</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B43" s="2" t="s">
         <v>48</v>
       </c>
       <c r="C43">
@@ -9792,7 +9791,7 @@
       <c r="A44" t="s">
         <v>140</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="2" t="s">
         <v>51</v>
       </c>
       <c r="C44">
@@ -9830,7 +9829,7 @@
       <c r="A45" t="s">
         <v>141</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="B45" s="2" t="s">
         <v>53</v>
       </c>
       <c r="C45">
@@ -9868,7 +9867,7 @@
       <c r="A46" t="s">
         <v>142</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="B46" s="2" t="s">
         <v>143</v>
       </c>
       <c r="C46">
@@ -9906,7 +9905,7 @@
       <c r="A47" t="s">
         <v>144</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="B47" s="2" t="s">
         <v>53</v>
       </c>
       <c r="C47">
@@ -9947,7 +9946,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A39:K43 A1:K36 A37:C37 G37:J37 A44:A45 C44:K45 A46:G46 I46 K46" numberStoredAsText="1"/>
+    <ignoredError sqref="K46 I46 A46:G46 C44:K45 A44:A45 G37:J37 A37:C37 A1:K36 A39:K43" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9956,7 +9955,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L47"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.6666666666667" customWidth="1"/>
     <col min="2" max="2" width="17.25" customWidth="1"/>
@@ -11537,7 +11536,7 @@
       <c r="G46">
         <v>100</v>
       </c>
-      <c r="H46" s="2" t="s">
+      <c r="H46" s="1" t="s">
         <v>31</v>
       </c>
       <c r="I46" t="s">
@@ -11575,7 +11574,7 @@
       <c r="G47">
         <v>50</v>
       </c>
-      <c r="H47" s="2" t="s">
+      <c r="H47" s="1" t="s">
         <v>31</v>
       </c>
       <c r="I47" t="s">
@@ -11592,13 +11591,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:K46" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:K47" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A39:K45 A1:K37 A46:G46 I46:K46 A48:K201" numberStoredAsText="1"/>
+    <ignoredError sqref="A48:K201 I46:K46 A46:G46 A1:K37 A39:K45" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11607,7 +11606,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L46"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.6666666666667" customWidth="1"/>
     <col min="2" max="2" width="17.25" customWidth="1"/>
@@ -12562,7 +12561,7 @@
         <v>31</v>
       </c>
       <c r="I28" t="s">
-        <v>116</v>
+        <v>5</v>
       </c>
       <c r="J28" t="s">
         <v>15</v>
@@ -12594,7 +12593,7 @@
         <v>31</v>
       </c>
       <c r="I29" t="s">
-        <v>116</v>
+        <v>5</v>
       </c>
       <c r="J29" t="s">
         <v>18</v>
@@ -12626,7 +12625,7 @@
         <v>31</v>
       </c>
       <c r="I30" t="s">
-        <v>116</v>
+        <v>5</v>
       </c>
       <c r="J30" t="s">
         <v>19</v>
@@ -12658,7 +12657,7 @@
         <v>31</v>
       </c>
       <c r="I31" t="s">
-        <v>116</v>
+        <v>5</v>
       </c>
       <c r="J31" t="s">
         <v>20</v>
@@ -13211,7 +13210,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A45:G45 A1:K44 I45:K45" numberStoredAsText="1"/>
+    <ignoredError sqref="I45:K45 A1:K27 A28:H31 J28:K31 A32:K44 A45:G45" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -13220,7 +13219,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L45"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.6666666666667" customWidth="1"/>
     <col min="2" max="2" width="22.75" customWidth="1"/>

</xml_diff>